<commit_message>
Fixing small issues in budget
</commit_message>
<xml_diff>
--- a/TFG-BUDGET.xlsx
+++ b/TFG-BUDGET.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pelay\Documents\EII\4º Software\TFG\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3FAE5BF6-7BFD-415B-8AFE-04E9E1384C3A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CBF0EBA2-AB4B-410E-BE0B-15C10ADF6B19}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{A8D38629-4F70-4F81-96AE-30B7AB9DB742}"/>
+    <workbookView xWindow="-19310" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="1" xr2:uid="{A8D38629-4F70-4F81-96AE-30B7AB9DB742}"/>
   </bookViews>
   <sheets>
     <sheet name="Company Definition" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="403" uniqueCount="159">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="404" uniqueCount="160">
   <si>
     <t>Microsoft Windows 11</t>
   </si>
@@ -223,9 +223,6 @@
     <t>Billing based on productive hours</t>
   </si>
   <si>
-    <t>BUDGET</t>
-  </si>
-  <si>
     <t>Overhead</t>
   </si>
   <si>
@@ -512,6 +509,12 @@
   </si>
   <si>
     <t>Total (+ VAT)</t>
+  </si>
+  <si>
+    <t>DETAILED BUDGET &amp; CLIENT BUDGET</t>
+  </si>
+  <si>
+    <t>COMPANY DEFINITION</t>
   </si>
 </sst>
 </file>
@@ -645,7 +648,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="13">
+  <borders count="14">
     <border>
       <left/>
       <right/>
@@ -799,6 +802,15 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -806,7 +818,7 @@
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="89">
+  <cellXfs count="93">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -966,18 +978,6 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="44" fontId="0" fillId="3" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="44" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="49" fontId="0" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -996,6 +996,24 @@
     <xf numFmtId="44" fontId="0" fillId="11" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="44" fontId="2" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="0" fillId="7" borderId="13" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="13" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="Comma" xfId="1" builtinId="3"/>
@@ -1336,7 +1354,7 @@
   <sheetData>
     <row r="1" spans="1:19" s="49" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="48" t="s">
-        <v>62</v>
+        <v>159</v>
       </c>
     </row>
     <row r="3" spans="1:19" x14ac:dyDescent="0.25">
@@ -1584,12 +1602,12 @@
       <c r="H8" s="5">
         <v>0</v>
       </c>
-      <c r="J8" s="74" t="s">
+      <c r="J8" s="89" t="s">
         <v>16</v>
       </c>
-      <c r="K8" s="74"/>
-      <c r="L8" s="74"/>
-      <c r="M8" s="74"/>
+      <c r="K8" s="89"/>
+      <c r="L8" s="89"/>
+      <c r="M8" s="89"/>
       <c r="N8" s="11">
         <f>SUM(N4:N7)</f>
         <v>207950.6</v>
@@ -1905,23 +1923,23 @@
       </c>
     </row>
     <row r="15" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="74" t="s">
+      <c r="A15" s="89" t="s">
         <v>16</v>
       </c>
-      <c r="B15" s="74"/>
-      <c r="C15" s="74"/>
-      <c r="D15" s="74"/>
+      <c r="B15" s="89"/>
+      <c r="C15" s="89"/>
+      <c r="D15" s="89"/>
       <c r="E15" s="47">
         <f>SUM(E4:E14)</f>
         <v>1502.7550000000001</v>
       </c>
       <c r="F15" s="12"/>
       <c r="H15" s="1"/>
-      <c r="J15" s="71" t="s">
+      <c r="J15" s="90" t="s">
         <v>16</v>
       </c>
-      <c r="K15" s="72"/>
-      <c r="L15" s="72"/>
+      <c r="K15" s="91"/>
+      <c r="L15" s="91"/>
       <c r="M15" s="17">
         <f>SUM(M11:M14)</f>
         <v>122959.22</v>
@@ -1967,9 +1985,9 @@
         <v>30</v>
       </c>
       <c r="R17" s="9" t="s">
-        <v>64</v>
-      </c>
-      <c r="S17" s="5">
+        <v>63</v>
+      </c>
+      <c r="S17" s="14">
         <f>((S16-S15)/S15)*100</f>
         <v>0</v>
       </c>
@@ -2166,7 +2184,7 @@
         <v>2400</v>
       </c>
       <c r="M25" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="N25" s="1">
         <f>S12/K22</f>
@@ -2277,75 +2295,78 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{11539845-83DD-446A-82A9-487B928930E4}">
-  <dimension ref="B1:O121"/>
+  <dimension ref="A1:O121"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="4" width="9.140625" style="53"/>
-    <col min="5" max="5" width="39" style="54" customWidth="1"/>
+    <col min="5" max="5" width="39" customWidth="1"/>
     <col min="6" max="6" width="16.140625" style="52" customWidth="1"/>
     <col min="8" max="8" width="12" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="14.5703125" customWidth="1"/>
-    <col min="10" max="10" width="12.140625" customWidth="1"/>
+    <col min="10" max="10" width="13.5703125" customWidth="1"/>
     <col min="13" max="13" width="50.140625" customWidth="1"/>
     <col min="14" max="14" width="21" customWidth="1"/>
     <col min="15" max="15" width="14" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="E1"/>
-    </row>
-    <row r="2" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="E2"/>
-    </row>
-    <row r="3" spans="2:15" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:15" s="86" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="88" t="s">
+        <v>158</v>
+      </c>
+      <c r="B1" s="85"/>
+      <c r="C1" s="85"/>
+      <c r="D1" s="85"/>
+      <c r="F1" s="87"/>
+    </row>
+    <row r="3" spans="1:15" x14ac:dyDescent="0.25">
       <c r="B3" s="8" t="s">
+        <v>64</v>
+      </c>
+      <c r="C3" s="8" t="s">
         <v>65</v>
       </c>
-      <c r="C3" s="8" t="s">
+      <c r="D3" s="8" t="s">
         <v>66</v>
       </c>
-      <c r="D3" s="8" t="s">
+      <c r="E3" s="8" t="s">
         <v>67</v>
-      </c>
-      <c r="E3" s="8" t="s">
-        <v>68</v>
       </c>
       <c r="F3" s="8" t="s">
         <v>5</v>
       </c>
       <c r="G3" s="8" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="H3" s="8" t="s">
         <v>49</v>
       </c>
       <c r="I3" s="8" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="J3" s="8" t="s">
         <v>16</v>
       </c>
       <c r="M3" s="8" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="N3" s="8" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="4" spans="2:15" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:15" x14ac:dyDescent="0.25">
       <c r="B4" s="61" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="C4" s="61"/>
       <c r="D4" s="61"/>
       <c r="E4" s="62" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="F4" s="63">
         <v>106</v>
       </c>
       <c r="G4" s="64" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="H4" s="65"/>
       <c r="I4" s="64"/>
@@ -2357,26 +2378,26 @@
         <f>E4</f>
         <v>Sprint 1: Analysis and planning</v>
       </c>
-      <c r="N4" s="75">
+      <c r="N4" s="71">
         <f>J4*1.25</f>
         <v>6777.2238571428579</v>
       </c>
-      <c r="O4" s="81"/>
-    </row>
-    <row r="5" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="O4" s="77"/>
+    </row>
+    <row r="5" spans="1:15" x14ac:dyDescent="0.25">
       <c r="B5" s="56"/>
       <c r="C5" s="56" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="D5" s="56"/>
       <c r="E5" s="55" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="F5" s="4">
         <v>8</v>
       </c>
       <c r="G5" s="54" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="H5" s="57"/>
       <c r="I5" s="58">
@@ -2384,28 +2405,28 @@
         <v>456.85414123989221</v>
       </c>
       <c r="J5" s="54"/>
-      <c r="M5" s="79" t="str">
+      <c r="M5" s="75" t="str">
         <f>E29</f>
         <v>Sprint 2: System design</v>
       </c>
-      <c r="N5" s="82">
+      <c r="N5" s="78">
         <f>J29*1.25</f>
         <v>5309.7035384097035</v>
       </c>
-      <c r="O5" s="81"/>
-    </row>
-    <row r="6" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="O5" s="77"/>
+    </row>
+    <row r="6" spans="1:15" x14ac:dyDescent="0.25">
       <c r="B6" s="66"/>
       <c r="C6" s="66"/>
       <c r="D6" s="66" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="E6" s="67" t="s">
         <v>17</v>
       </c>
       <c r="F6" s="6"/>
       <c r="G6" s="68" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="H6" s="69">
         <f>'Company Definition'!N$18</f>
@@ -2417,26 +2438,26 @@
         <f>E46</f>
         <v>Sprint 3: Backend &amp; pipeline development</v>
       </c>
-      <c r="N6" s="75">
+      <c r="N6" s="71">
         <f>J46*1.25</f>
         <v>4095.7911199460923</v>
       </c>
-      <c r="O6" s="81"/>
-    </row>
-    <row r="7" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="O6" s="77"/>
+    </row>
+    <row r="7" spans="1:15" x14ac:dyDescent="0.25">
       <c r="B7" s="56"/>
       <c r="C7" s="56" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="D7" s="56"/>
       <c r="E7" s="55" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="F7" s="4">
         <v>8</v>
       </c>
       <c r="G7" s="54" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="H7" s="57"/>
       <c r="I7" s="58">
@@ -2444,28 +2465,28 @@
         <v>456.85414123989221</v>
       </c>
       <c r="J7" s="54"/>
-      <c r="M7" s="79" t="str">
+      <c r="M7" s="75" t="str">
         <f>E59</f>
         <v>Sprint 4: Full NLP pipeline implementation</v>
       </c>
-      <c r="N7" s="82">
+      <c r="N7" s="78">
         <f>J59*1.25</f>
         <v>4622.4773679245291</v>
       </c>
-      <c r="O7" s="81"/>
-    </row>
-    <row r="8" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="O7" s="77"/>
+    </row>
+    <row r="8" spans="1:15" x14ac:dyDescent="0.25">
       <c r="B8" s="66"/>
       <c r="C8" s="66"/>
       <c r="D8" s="66" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="E8" s="67" t="s">
         <v>17</v>
       </c>
       <c r="F8" s="6"/>
       <c r="G8" s="68" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="H8" s="69">
         <f>'Company Definition'!N$18</f>
@@ -2477,26 +2498,26 @@
         <f>E76</f>
         <v>Sprint 5: Data visualizations and web application aspects</v>
       </c>
-      <c r="N8" s="75">
+      <c r="N8" s="71">
         <f>J76*1.25</f>
         <v>3918.0629272237193</v>
       </c>
-      <c r="O8" s="81"/>
-    </row>
-    <row r="9" spans="2:15" ht="30" x14ac:dyDescent="0.25">
+      <c r="O8" s="77"/>
+    </row>
+    <row r="9" spans="1:15" ht="30" x14ac:dyDescent="0.25">
       <c r="B9" s="56"/>
       <c r="C9" s="56" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="D9" s="56"/>
       <c r="E9" s="55" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="F9" s="4">
         <v>10</v>
       </c>
       <c r="G9" s="54" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="H9" s="57"/>
       <c r="I9" s="58">
@@ -2504,28 +2525,28 @@
         <v>571.06767654986527</v>
       </c>
       <c r="J9" s="54"/>
-      <c r="M9" s="79" t="str">
+      <c r="M9" s="75" t="str">
         <f>E89</f>
         <v>Sprint 6: Final documentation &amp; product refinements</v>
       </c>
-      <c r="N9" s="82">
+      <c r="N9" s="78">
         <f>J89*1.25</f>
         <v>2216.7987614555254</v>
       </c>
-      <c r="O9" s="81"/>
-    </row>
-    <row r="10" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="O9" s="77"/>
+    </row>
+    <row r="10" spans="1:15" x14ac:dyDescent="0.25">
       <c r="B10" s="66"/>
       <c r="C10" s="66"/>
       <c r="D10" s="66" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="E10" s="67" t="s">
         <v>17</v>
       </c>
       <c r="F10" s="6"/>
       <c r="G10" s="68" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="H10" s="69">
         <f>'Company Definition'!N$18</f>
@@ -2534,28 +2555,28 @@
       <c r="I10" s="68"/>
       <c r="J10" s="68"/>
       <c r="M10" s="68" t="s">
-        <v>156</v>
-      </c>
-      <c r="N10" s="75">
+        <v>155</v>
+      </c>
+      <c r="N10" s="71">
         <f>J96*1.25</f>
         <v>4425.7290889487876</v>
       </c>
-      <c r="O10" s="81"/>
-    </row>
-    <row r="11" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="O10" s="77"/>
+    </row>
+    <row r="11" spans="1:15" x14ac:dyDescent="0.25">
       <c r="B11" s="56"/>
       <c r="C11" s="56" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="D11" s="56"/>
       <c r="E11" s="55" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="F11" s="4">
         <v>10</v>
       </c>
       <c r="G11" s="54" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="H11" s="57"/>
       <c r="I11" s="58">
@@ -2563,26 +2584,26 @@
         <v>571.06767654986527</v>
       </c>
       <c r="J11" s="54"/>
-      <c r="M11" s="83" t="s">
-        <v>136</v>
-      </c>
-      <c r="N11" s="84">
+      <c r="M11" s="79" t="s">
+        <v>135</v>
+      </c>
+      <c r="N11" s="80">
         <f>SUM(N4:N10)</f>
         <v>31365.786661051214</v>
       </c>
     </row>
-    <row r="12" spans="2:15" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:15" x14ac:dyDescent="0.25">
       <c r="B12" s="66"/>
       <c r="C12" s="66"/>
       <c r="D12" s="66" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="E12" s="67" t="s">
         <v>17</v>
       </c>
       <c r="F12" s="6"/>
       <c r="G12" s="68" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="H12" s="69">
         <f>'Company Definition'!N$18</f>
@@ -2590,28 +2611,28 @@
       </c>
       <c r="I12" s="68"/>
       <c r="J12" s="68"/>
-      <c r="M12" s="85" t="s">
-        <v>157</v>
-      </c>
-      <c r="N12" s="86">
+      <c r="M12" s="81" t="s">
+        <v>156</v>
+      </c>
+      <c r="N12" s="82">
         <f>N11*0.21</f>
         <v>6586.8151988207546</v>
       </c>
     </row>
-    <row r="13" spans="2:15" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:15" x14ac:dyDescent="0.25">
       <c r="B13" s="56"/>
       <c r="C13" s="56" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="D13" s="56"/>
       <c r="E13" s="55" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="F13" s="4">
         <v>10</v>
       </c>
       <c r="G13" s="54" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="H13" s="57"/>
       <c r="I13" s="58">
@@ -2619,26 +2640,26 @@
         <v>571.06767654986527</v>
       </c>
       <c r="J13" s="54"/>
-      <c r="M13" s="87" t="s">
-        <v>158</v>
-      </c>
-      <c r="N13" s="88">
+      <c r="M13" s="83" t="s">
+        <v>157</v>
+      </c>
+      <c r="N13" s="84">
         <f>N11*1.21</f>
         <v>37952.601859871967</v>
       </c>
     </row>
-    <row r="14" spans="2:15" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:15" ht="12" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B14" s="66"/>
       <c r="C14" s="66"/>
       <c r="D14" s="66" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="E14" s="67" t="s">
         <v>17</v>
       </c>
       <c r="F14" s="6"/>
       <c r="G14" s="68" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="H14" s="69">
         <f>'Company Definition'!N$18</f>
@@ -2646,22 +2667,22 @@
       </c>
       <c r="I14" s="68"/>
       <c r="J14" s="68"/>
-      <c r="N14" s="81"/>
-    </row>
-    <row r="15" spans="2:15" ht="32.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="N14" s="77"/>
+    </row>
+    <row r="15" spans="1:15" ht="32.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B15" s="56"/>
       <c r="C15" s="56" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="D15" s="56"/>
       <c r="E15" s="55" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="F15" s="4">
         <v>8</v>
       </c>
       <c r="G15" s="54" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="H15" s="57"/>
       <c r="I15" s="58">
@@ -2670,18 +2691,18 @@
       </c>
       <c r="J15" s="54"/>
     </row>
-    <row r="16" spans="2:15" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:15" x14ac:dyDescent="0.25">
       <c r="B16" s="66"/>
       <c r="C16" s="66"/>
       <c r="D16" s="66" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="E16" s="67" t="s">
         <v>18</v>
       </c>
       <c r="F16" s="6"/>
       <c r="G16" s="68" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="H16" s="69">
         <f>'Company Definition'!N$19</f>
@@ -2693,17 +2714,17 @@
     <row r="17" spans="2:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B17" s="56"/>
       <c r="C17" s="56" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="D17" s="56"/>
       <c r="E17" s="55" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="F17" s="4">
         <v>8</v>
       </c>
       <c r="G17" s="54" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="H17" s="57"/>
       <c r="I17" s="58">
@@ -2716,14 +2737,14 @@
       <c r="B18" s="66"/>
       <c r="C18" s="66"/>
       <c r="D18" s="66" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="E18" s="67" t="s">
         <v>19</v>
       </c>
       <c r="F18" s="6"/>
       <c r="G18" s="68" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="H18" s="69">
         <f>'Company Definition'!N$20</f>
@@ -2735,17 +2756,17 @@
     <row r="19" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B19" s="56"/>
       <c r="C19" s="56" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="D19" s="56"/>
       <c r="E19" s="55" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="F19" s="4">
         <v>8</v>
       </c>
       <c r="G19" s="54" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="H19" s="57"/>
       <c r="I19" s="58">
@@ -2758,14 +2779,14 @@
       <c r="B20" s="66"/>
       <c r="C20" s="66"/>
       <c r="D20" s="66" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="E20" s="67" t="s">
         <v>19</v>
       </c>
       <c r="F20" s="6"/>
       <c r="G20" s="68" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="H20" s="69">
         <f>'Company Definition'!N$20</f>
@@ -2777,17 +2798,17 @@
     <row r="21" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B21" s="56"/>
       <c r="C21" s="56" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="D21" s="56"/>
       <c r="E21" s="55" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="F21" s="4">
         <v>8</v>
       </c>
       <c r="G21" s="54" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="H21" s="57"/>
       <c r="I21" s="58">
@@ -2800,14 +2821,14 @@
       <c r="B22" s="66"/>
       <c r="C22" s="66"/>
       <c r="D22" s="66" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="E22" s="67" t="s">
         <v>17</v>
       </c>
       <c r="F22" s="6"/>
       <c r="G22" s="68" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="H22" s="69">
         <f>'Company Definition'!N$18</f>
@@ -2819,17 +2840,17 @@
     <row r="23" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B23" s="56"/>
       <c r="C23" s="56" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="D23" s="56"/>
       <c r="E23" s="55" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F23" s="4">
         <v>8</v>
       </c>
       <c r="G23" s="54" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="H23" s="57"/>
       <c r="I23" s="58">
@@ -2842,14 +2863,14 @@
       <c r="B24" s="66"/>
       <c r="C24" s="66"/>
       <c r="D24" s="66" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="E24" s="67" t="s">
         <v>17</v>
       </c>
       <c r="F24" s="6"/>
       <c r="G24" s="68" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="H24" s="69">
         <f>'Company Definition'!N$18</f>
@@ -2861,17 +2882,17 @@
     <row r="25" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B25" s="56"/>
       <c r="C25" s="56" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="D25" s="56"/>
       <c r="E25" s="55" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="F25" s="4">
         <v>8</v>
       </c>
       <c r="G25" s="54" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="H25" s="57"/>
       <c r="I25" s="58">
@@ -2884,14 +2905,14 @@
       <c r="B26" s="66"/>
       <c r="C26" s="66"/>
       <c r="D26" s="66" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="E26" s="67" t="s">
         <v>19</v>
       </c>
       <c r="F26" s="6"/>
       <c r="G26" s="68" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="H26" s="69">
         <f>'Company Definition'!N$20</f>
@@ -2903,17 +2924,17 @@
     <row r="27" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B27" s="56"/>
       <c r="C27" s="56" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="D27" s="56"/>
       <c r="E27" s="55" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="F27" s="4">
         <v>12</v>
       </c>
       <c r="G27" s="54" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="H27" s="57"/>
       <c r="I27" s="58">
@@ -2926,14 +2947,14 @@
       <c r="B28" s="66"/>
       <c r="C28" s="66"/>
       <c r="D28" s="66" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="E28" s="67" t="s">
         <v>19</v>
       </c>
       <c r="F28" s="6"/>
       <c r="G28" s="68" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="H28" s="69">
         <f>'Company Definition'!N$20</f>
@@ -2944,18 +2965,18 @@
     </row>
     <row r="29" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B29" s="61" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="C29" s="61"/>
       <c r="D29" s="61"/>
       <c r="E29" s="62" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="F29" s="63">
         <v>84</v>
       </c>
       <c r="G29" s="64" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="H29" s="65"/>
       <c r="I29" s="64"/>
@@ -2967,17 +2988,17 @@
     <row r="30" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B30" s="56"/>
       <c r="C30" s="56" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="D30" s="56"/>
       <c r="E30" s="55" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="F30" s="4">
         <v>8</v>
       </c>
       <c r="G30" s="54" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="H30" s="57"/>
       <c r="I30" s="58">
@@ -2990,14 +3011,14 @@
       <c r="B31" s="66"/>
       <c r="C31" s="66"/>
       <c r="D31" s="66" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="E31" s="67" t="s">
         <v>18</v>
       </c>
       <c r="F31" s="6"/>
       <c r="G31" s="68" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="H31" s="69">
         <f>'Company Definition'!N$19</f>
@@ -3009,17 +3030,17 @@
     <row r="32" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B32" s="56"/>
       <c r="C32" s="56" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="D32" s="56"/>
       <c r="E32" s="55" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="F32" s="4">
         <v>10</v>
       </c>
       <c r="G32" s="54" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="H32" s="57"/>
       <c r="I32" s="58">
@@ -3032,14 +3053,14 @@
       <c r="B33" s="66"/>
       <c r="C33" s="66"/>
       <c r="D33" s="66" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="E33" s="67" t="s">
         <v>17</v>
       </c>
       <c r="F33" s="6"/>
       <c r="G33" s="68" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="H33" s="69">
         <f>'Company Definition'!N$18</f>
@@ -3051,17 +3072,17 @@
     <row r="34" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B34" s="56"/>
       <c r="C34" s="56" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="D34" s="56"/>
       <c r="E34" s="55" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="F34" s="4">
         <v>12</v>
       </c>
       <c r="G34" s="54" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="H34" s="57"/>
       <c r="I34" s="58">
@@ -3073,17 +3094,17 @@
     <row r="35" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B35" s="66"/>
       <c r="C35" s="56" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="D35" s="66" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="E35" s="67" t="s">
         <v>17</v>
       </c>
       <c r="F35" s="6"/>
       <c r="G35" s="68" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="H35" s="69">
         <f>'Company Definition'!N$18</f>
@@ -3097,13 +3118,13 @@
       <c r="C36" s="66"/>
       <c r="D36" s="56"/>
       <c r="E36" s="55" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="F36" s="4">
         <v>8</v>
       </c>
       <c r="G36" s="54" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="H36" s="57"/>
       <c r="I36" s="58">
@@ -3115,17 +3136,17 @@
     <row r="37" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B37" s="66"/>
       <c r="C37" s="56" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="D37" s="66" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="E37" s="67" t="s">
         <v>18</v>
       </c>
       <c r="F37" s="6"/>
       <c r="G37" s="68" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="H37" s="69">
         <f>'Company Definition'!N$19</f>
@@ -3139,13 +3160,13 @@
       <c r="C38" s="66"/>
       <c r="D38" s="56"/>
       <c r="E38" s="55" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="F38" s="4">
         <v>10</v>
       </c>
       <c r="G38" s="54" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="H38" s="57"/>
       <c r="I38" s="58">
@@ -3157,17 +3178,17 @@
     <row r="39" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B39" s="66"/>
       <c r="C39" s="56" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="D39" s="66" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="E39" s="67" t="s">
         <v>17</v>
       </c>
       <c r="F39" s="6"/>
       <c r="G39" s="68" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="H39" s="69">
         <f>'Company Definition'!L$18</f>
@@ -3179,19 +3200,19 @@
     <row r="40" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B40" s="56"/>
       <c r="C40" s="56" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="D40" s="56" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="E40" s="55" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="F40" s="4">
         <v>6</v>
       </c>
       <c r="G40" s="54" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="H40" s="57"/>
       <c r="I40" s="58">
@@ -3209,7 +3230,7 @@
       </c>
       <c r="F41" s="6"/>
       <c r="G41" s="68" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="H41" s="69">
         <f>'Company Definition'!N$20</f>
@@ -3221,19 +3242,19 @@
     <row r="42" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B42" s="56"/>
       <c r="C42" s="56" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="D42" s="56" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="E42" s="55" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="F42" s="4">
         <v>20</v>
       </c>
       <c r="G42" s="54" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="H42" s="57"/>
       <c r="I42" s="58">
@@ -3251,7 +3272,7 @@
       </c>
       <c r="F43" s="6"/>
       <c r="G43" s="68" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="H43" s="69">
         <f>'Company Definition'!N$20</f>
@@ -3263,19 +3284,19 @@
     <row r="44" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B44" s="56"/>
       <c r="C44" s="56" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="D44" s="56" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="E44" s="55" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="F44" s="4">
         <v>10</v>
       </c>
       <c r="G44" s="54" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="H44" s="57"/>
       <c r="I44" s="58">
@@ -3293,7 +3314,7 @@
       </c>
       <c r="F45" s="6"/>
       <c r="G45" s="68" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="H45" s="69">
         <f>'Company Definition'!N$20</f>
@@ -3302,20 +3323,20 @@
       <c r="I45" s="68"/>
       <c r="J45" s="68"/>
     </row>
-    <row r="46" spans="2:10" ht="30" x14ac:dyDescent="0.25">
+    <row r="46" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B46" s="61" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C46" s="61"/>
       <c r="D46" s="61"/>
       <c r="E46" s="62" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="F46" s="63">
         <v>73</v>
       </c>
       <c r="G46" s="64" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="H46" s="65"/>
       <c r="I46" s="64"/>
@@ -3327,17 +3348,17 @@
     <row r="47" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B47" s="56"/>
       <c r="C47" s="56" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="D47" s="56"/>
       <c r="E47" s="55" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="F47" s="4">
         <v>8</v>
       </c>
       <c r="G47" s="54" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="H47" s="57"/>
       <c r="I47" s="58">
@@ -3350,14 +3371,14 @@
       <c r="B48" s="66"/>
       <c r="C48" s="66"/>
       <c r="D48" s="66" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="E48" s="67" t="s">
         <v>19</v>
       </c>
       <c r="F48" s="6"/>
       <c r="G48" s="68" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="H48" s="69">
         <f>'Company Definition'!N$20</f>
@@ -3369,17 +3390,17 @@
     <row r="49" spans="2:10" ht="30" x14ac:dyDescent="0.25">
       <c r="B49" s="56"/>
       <c r="C49" s="56" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="D49" s="56"/>
       <c r="E49" s="55" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="F49" s="4">
         <v>8</v>
       </c>
       <c r="G49" s="54" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="H49" s="57"/>
       <c r="I49" s="58">
@@ -3392,14 +3413,14 @@
       <c r="B50" s="66"/>
       <c r="C50" s="66"/>
       <c r="D50" s="66" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="E50" s="67" t="s">
         <v>18</v>
       </c>
       <c r="F50" s="6"/>
       <c r="G50" s="68" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="H50" s="69">
         <f>'Company Definition'!N$19</f>
@@ -3408,20 +3429,20 @@
       <c r="I50" s="68"/>
       <c r="J50" s="68"/>
     </row>
-    <row r="51" spans="2:10" ht="30" x14ac:dyDescent="0.25">
+    <row r="51" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B51" s="56"/>
       <c r="C51" s="56" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="D51" s="56"/>
       <c r="E51" s="55" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="F51" s="4">
         <v>10</v>
       </c>
       <c r="G51" s="54" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="H51" s="57"/>
       <c r="I51" s="58">
@@ -3434,14 +3455,14 @@
       <c r="B52" s="66"/>
       <c r="C52" s="66"/>
       <c r="D52" s="66" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="E52" s="67" t="s">
         <v>18</v>
       </c>
       <c r="F52" s="6"/>
       <c r="G52" s="68" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="H52" s="69">
         <f>'Company Definition'!N$19</f>
@@ -3453,17 +3474,17 @@
     <row r="53" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B53" s="56"/>
       <c r="C53" s="56" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="D53" s="56"/>
       <c r="E53" s="55" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="F53" s="4">
         <v>8</v>
       </c>
       <c r="G53" s="54" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="H53" s="57"/>
       <c r="I53" s="58">
@@ -3476,14 +3497,14 @@
       <c r="B54" s="66"/>
       <c r="C54" s="66"/>
       <c r="D54" s="66" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="E54" s="67" t="s">
         <v>19</v>
       </c>
       <c r="F54" s="6"/>
       <c r="G54" s="68" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="H54" s="69">
         <f>'Company Definition'!N$20</f>
@@ -3495,17 +3516,17 @@
     <row r="55" spans="2:10" ht="30" x14ac:dyDescent="0.25">
       <c r="B55" s="56"/>
       <c r="C55" s="56" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="D55" s="56"/>
       <c r="E55" s="55" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="F55" s="4">
         <v>14</v>
       </c>
       <c r="G55" s="54" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="H55" s="57"/>
       <c r="I55" s="58">
@@ -3518,14 +3539,14 @@
       <c r="B56" s="66"/>
       <c r="C56" s="66"/>
       <c r="D56" s="66" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="E56" s="67" t="s">
         <v>18</v>
       </c>
       <c r="F56" s="6"/>
       <c r="G56" s="68" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="H56" s="69">
         <f>'Company Definition'!N$19</f>
@@ -3537,19 +3558,19 @@
     <row r="57" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B57" s="56"/>
       <c r="C57" s="56" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="D57" s="56" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="E57" s="55" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="F57" s="4">
         <v>25</v>
       </c>
       <c r="G57" s="54" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="H57" s="57"/>
       <c r="I57" s="58">
@@ -3567,7 +3588,7 @@
       </c>
       <c r="F58" s="6"/>
       <c r="G58" s="68" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="H58" s="69">
         <f>'Company Definition'!N$20</f>
@@ -3576,20 +3597,20 @@
       <c r="I58" s="68"/>
       <c r="J58" s="68"/>
     </row>
-    <row r="59" spans="2:10" ht="30" x14ac:dyDescent="0.25">
+    <row r="59" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B59" s="61" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="C59" s="61"/>
       <c r="D59" s="61"/>
       <c r="E59" s="62" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="F59" s="63">
         <v>81</v>
       </c>
       <c r="G59" s="64" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="H59" s="65"/>
       <c r="I59" s="64"/>
@@ -3601,17 +3622,17 @@
     <row r="60" spans="2:10" ht="30" x14ac:dyDescent="0.25">
       <c r="B60" s="56"/>
       <c r="C60" s="56" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="D60" s="56"/>
       <c r="E60" s="55" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="F60" s="4">
         <v>6</v>
       </c>
       <c r="G60" s="54" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="H60" s="57"/>
       <c r="I60" s="58">
@@ -3624,14 +3645,14 @@
       <c r="B61" s="66"/>
       <c r="C61" s="66"/>
       <c r="D61" s="66" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="E61" s="67" t="s">
         <v>18</v>
       </c>
       <c r="F61" s="6"/>
       <c r="G61" s="68" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="H61" s="69">
         <f>'Company Definition'!N$19</f>
@@ -3643,11 +3664,11 @@
     <row r="62" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B62" s="56"/>
       <c r="C62" s="56" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="D62" s="56"/>
       <c r="E62" s="55" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="F62" s="4">
         <v>12</v>
@@ -3664,7 +3685,7 @@
       <c r="B63" s="66"/>
       <c r="C63" s="66"/>
       <c r="D63" s="66" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="E63" s="67" t="s">
         <v>18</v>
@@ -3681,11 +3702,11 @@
     <row r="64" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B64" s="56"/>
       <c r="C64" s="56" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="D64" s="56"/>
       <c r="E64" s="55" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="F64" s="4">
         <v>8</v>
@@ -3702,7 +3723,7 @@
       <c r="B65" s="66"/>
       <c r="C65" s="66"/>
       <c r="D65" s="66" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="E65" s="67" t="s">
         <v>19</v>
@@ -3716,14 +3737,14 @@
       <c r="I65" s="68"/>
       <c r="J65" s="68"/>
     </row>
-    <row r="66" spans="2:10" ht="30" x14ac:dyDescent="0.25">
+    <row r="66" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B66" s="56"/>
       <c r="C66" s="56" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="D66" s="56"/>
       <c r="E66" s="55" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="F66" s="4">
         <v>4</v>
@@ -3740,7 +3761,7 @@
       <c r="B67" s="66"/>
       <c r="C67" s="66"/>
       <c r="D67" s="66" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="E67" s="67" t="s">
         <v>19</v>
@@ -3757,11 +3778,11 @@
     <row r="68" spans="2:10" ht="30" x14ac:dyDescent="0.25">
       <c r="B68" s="56"/>
       <c r="C68" s="56" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="D68" s="56"/>
       <c r="E68" s="55" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="F68" s="4">
         <v>10</v>
@@ -3778,7 +3799,7 @@
       <c r="B69" s="66"/>
       <c r="C69" s="66"/>
       <c r="D69" s="66" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="E69" s="67" t="s">
         <v>18</v>
@@ -3795,11 +3816,11 @@
     <row r="70" spans="2:10" ht="30" x14ac:dyDescent="0.25">
       <c r="B70" s="56"/>
       <c r="C70" s="56" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="D70" s="56"/>
       <c r="E70" s="55" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="F70" s="4">
         <v>15</v>
@@ -3816,7 +3837,7 @@
       <c r="B71" s="66"/>
       <c r="C71" s="66"/>
       <c r="D71" s="66" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="E71" s="67" t="s">
         <v>18</v>
@@ -3833,11 +3854,11 @@
     <row r="72" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B72" s="56"/>
       <c r="C72" s="56" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="D72" s="56"/>
       <c r="E72" s="55" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="F72" s="4">
         <v>10</v>
@@ -3854,7 +3875,7 @@
       <c r="B73" s="66"/>
       <c r="C73" s="66"/>
       <c r="D73" s="66" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="E73" s="67" t="s">
         <v>19</v>
@@ -3871,11 +3892,11 @@
     <row r="74" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B74" s="56"/>
       <c r="C74" s="56" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="D74" s="56"/>
       <c r="E74" s="55" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="F74" s="4">
         <v>16</v>
@@ -3892,7 +3913,7 @@
       <c r="B75" s="66"/>
       <c r="C75" s="66"/>
       <c r="D75" s="66" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="E75" s="67" t="s">
         <v>19</v>
@@ -3908,12 +3929,12 @@
     </row>
     <row r="76" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B76" s="61" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C76" s="61"/>
       <c r="D76" s="61"/>
       <c r="E76" s="70" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="F76" s="63">
         <v>76</v>
@@ -3929,11 +3950,11 @@
     <row r="77" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B77" s="56"/>
       <c r="C77" s="56" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="D77" s="56"/>
       <c r="E77" s="55" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="F77" s="4">
         <v>8</v>
@@ -3950,7 +3971,7 @@
       <c r="B78" s="66"/>
       <c r="C78" s="66"/>
       <c r="D78" s="66" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="E78" s="67" t="s">
         <v>19</v>
@@ -3967,11 +3988,11 @@
     <row r="79" spans="2:10" ht="30" x14ac:dyDescent="0.25">
       <c r="B79" s="56"/>
       <c r="C79" s="56" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="D79" s="56"/>
       <c r="E79" s="55" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="F79" s="4">
         <v>10</v>
@@ -3988,7 +4009,7 @@
       <c r="B80" s="66"/>
       <c r="C80" s="66"/>
       <c r="D80" s="66" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="E80" s="67" t="s">
         <v>19</v>
@@ -4005,11 +4026,11 @@
     <row r="81" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B81" s="56"/>
       <c r="C81" s="56" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="D81" s="56"/>
       <c r="E81" s="55" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="F81" s="4">
         <v>15</v>
@@ -4026,7 +4047,7 @@
       <c r="B82" s="66"/>
       <c r="C82" s="66"/>
       <c r="D82" s="66" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="E82" s="67" t="s">
         <v>19</v>
@@ -4043,11 +4064,11 @@
     <row r="83" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B83" s="56"/>
       <c r="C83" s="56" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="D83" s="56"/>
       <c r="E83" s="55" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="F83" s="4">
         <v>10</v>
@@ -4064,7 +4085,7 @@
       <c r="B84" s="66"/>
       <c r="C84" s="66"/>
       <c r="D84" s="66" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="E84" s="67" t="s">
         <v>19</v>
@@ -4081,11 +4102,11 @@
     <row r="85" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B85" s="56"/>
       <c r="C85" s="56" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="D85" s="56"/>
       <c r="E85" s="55" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="F85" s="4">
         <v>8</v>
@@ -4102,7 +4123,7 @@
       <c r="B86" s="66"/>
       <c r="C86" s="66"/>
       <c r="D86" s="66" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="E86" s="67" t="s">
         <v>19</v>
@@ -4119,11 +4140,11 @@
     <row r="87" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B87" s="56"/>
       <c r="C87" s="56" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="D87" s="56"/>
       <c r="E87" s="55" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="F87" s="4">
         <v>25</v>
@@ -4140,7 +4161,7 @@
       <c r="B88" s="66"/>
       <c r="C88" s="66"/>
       <c r="D88" s="66" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="E88" s="67" t="s">
         <v>19</v>
@@ -4156,12 +4177,12 @@
     </row>
     <row r="89" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B89" s="61" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="C89" s="61"/>
       <c r="D89" s="61"/>
       <c r="E89" s="70" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="F89" s="63">
         <v>43</v>
@@ -4177,11 +4198,11 @@
     <row r="90" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B90" s="56"/>
       <c r="C90" s="56" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="D90" s="56"/>
       <c r="E90" s="55" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="F90" s="4">
         <v>25</v>
@@ -4198,7 +4219,7 @@
       <c r="B91" s="66"/>
       <c r="C91" s="66"/>
       <c r="D91" s="66" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="E91" s="67" t="s">
         <v>19</v>
@@ -4215,11 +4236,11 @@
     <row r="92" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B92" s="56"/>
       <c r="C92" s="56" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="D92" s="56"/>
       <c r="E92" s="55" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="F92" s="4">
         <v>10</v>
@@ -4236,7 +4257,7 @@
       <c r="B93" s="66"/>
       <c r="C93" s="66"/>
       <c r="D93" s="66" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="E93" s="67" t="s">
         <v>19</v>
@@ -4253,11 +4274,11 @@
     <row r="94" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B94" s="56"/>
       <c r="C94" s="56" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="D94" s="56"/>
       <c r="E94" s="55" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="F94" s="4">
         <v>8</v>
@@ -4274,7 +4295,7 @@
       <c r="B95" s="66"/>
       <c r="C95" s="66"/>
       <c r="D95" s="66" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="E95" s="67" t="s">
         <v>19</v>
@@ -4290,12 +4311,12 @@
     </row>
     <row r="96" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B96" s="61" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="C96" s="61"/>
       <c r="D96" s="61"/>
       <c r="E96" s="70" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="F96" s="63">
         <v>8</v>
@@ -4311,46 +4332,46 @@
     <row r="97" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B97" s="66"/>
       <c r="C97" s="66" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="D97" s="66"/>
       <c r="E97" s="67" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="F97" s="6">
         <v>1</v>
       </c>
       <c r="G97" s="68"/>
       <c r="H97" s="69"/>
-      <c r="I97" s="75">
+      <c r="I97" s="71">
         <f>(H98+H99)*F97</f>
         <v>98.349535309973049</v>
       </c>
       <c r="J97" s="68"/>
     </row>
     <row r="98" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B98" s="76"/>
-      <c r="C98" s="76"/>
-      <c r="D98" s="76" t="s">
-        <v>79</v>
-      </c>
-      <c r="E98" s="77" t="s">
+      <c r="B98" s="72"/>
+      <c r="C98" s="72"/>
+      <c r="D98" s="72" t="s">
+        <v>78</v>
+      </c>
+      <c r="E98" s="73" t="s">
         <v>19</v>
       </c>
-      <c r="F98" s="78"/>
-      <c r="G98" s="79"/>
-      <c r="H98" s="80">
+      <c r="F98" s="74"/>
+      <c r="G98" s="75"/>
+      <c r="H98" s="76">
         <f>'Company Definition'!N$20</f>
         <v>41.242767654986523</v>
       </c>
-      <c r="I98" s="79"/>
-      <c r="J98" s="79"/>
+      <c r="I98" s="75"/>
+      <c r="J98" s="75"/>
     </row>
     <row r="99" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B99" s="56"/>
       <c r="C99" s="56"/>
       <c r="D99" s="56" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="E99" s="55" t="s">
         <v>20</v>
@@ -4367,46 +4388,46 @@
     <row r="100" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B100" s="66"/>
       <c r="C100" s="66" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="D100" s="66"/>
       <c r="E100" s="67" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="F100" s="6">
         <v>2</v>
       </c>
       <c r="G100" s="68"/>
       <c r="H100" s="69"/>
-      <c r="I100" s="75">
+      <c r="I100" s="71">
         <f t="shared" ref="I100" si="29">(H101+H102)*F100</f>
         <v>196.6990706199461</v>
       </c>
       <c r="J100" s="68"/>
     </row>
     <row r="101" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B101" s="76"/>
-      <c r="C101" s="76"/>
-      <c r="D101" s="76" t="s">
-        <v>81</v>
-      </c>
-      <c r="E101" s="77" t="s">
+      <c r="B101" s="72"/>
+      <c r="C101" s="72"/>
+      <c r="D101" s="72" t="s">
+        <v>80</v>
+      </c>
+      <c r="E101" s="73" t="s">
         <v>19</v>
       </c>
-      <c r="F101" s="78"/>
-      <c r="G101" s="79"/>
-      <c r="H101" s="80">
+      <c r="F101" s="74"/>
+      <c r="G101" s="75"/>
+      <c r="H101" s="76">
         <f>'Company Definition'!N$20</f>
         <v>41.242767654986523</v>
       </c>
-      <c r="I101" s="79"/>
-      <c r="J101" s="79"/>
+      <c r="I101" s="75"/>
+      <c r="J101" s="75"/>
     </row>
     <row r="102" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B102" s="56"/>
       <c r="C102" s="56"/>
       <c r="D102" s="56" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="E102" s="55" t="s">
         <v>20</v>
@@ -4423,46 +4444,46 @@
     <row r="103" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B103" s="66"/>
       <c r="C103" s="66" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="D103" s="66"/>
       <c r="E103" s="67" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="F103" s="6">
         <v>3</v>
       </c>
       <c r="G103" s="68"/>
       <c r="H103" s="69"/>
-      <c r="I103" s="75">
+      <c r="I103" s="71">
         <f t="shared" ref="I103" si="30">(H104+H105)*F103</f>
         <v>295.04860592991918</v>
       </c>
       <c r="J103" s="68"/>
     </row>
     <row r="104" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B104" s="76"/>
-      <c r="C104" s="76"/>
-      <c r="D104" s="76" t="s">
-        <v>126</v>
-      </c>
-      <c r="E104" s="77" t="s">
+      <c r="B104" s="72"/>
+      <c r="C104" s="72"/>
+      <c r="D104" s="72" t="s">
+        <v>125</v>
+      </c>
+      <c r="E104" s="73" t="s">
         <v>19</v>
       </c>
-      <c r="F104" s="78"/>
-      <c r="G104" s="79"/>
-      <c r="H104" s="80">
+      <c r="F104" s="74"/>
+      <c r="G104" s="75"/>
+      <c r="H104" s="76">
         <f>'Company Definition'!N$20</f>
         <v>41.242767654986523</v>
       </c>
-      <c r="I104" s="79"/>
-      <c r="J104" s="79"/>
+      <c r="I104" s="75"/>
+      <c r="J104" s="75"/>
     </row>
     <row r="105" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B105" s="56"/>
       <c r="C105" s="56"/>
       <c r="D105" s="56" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="E105" s="55" t="s">
         <v>20</v>
@@ -4479,46 +4500,46 @@
     <row r="106" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B106" s="66"/>
       <c r="C106" s="66" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="D106" s="66"/>
       <c r="E106" s="67" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="F106" s="6">
         <v>4</v>
       </c>
       <c r="G106" s="68"/>
       <c r="H106" s="69"/>
-      <c r="I106" s="75">
+      <c r="I106" s="71">
         <f t="shared" ref="I106" si="31">(H107+H108)*F106</f>
         <v>393.3981412398922</v>
       </c>
       <c r="J106" s="68"/>
     </row>
     <row r="107" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B107" s="76"/>
-      <c r="C107" s="76"/>
-      <c r="D107" s="76" t="s">
-        <v>128</v>
-      </c>
-      <c r="E107" s="77" t="s">
+      <c r="B107" s="72"/>
+      <c r="C107" s="72"/>
+      <c r="D107" s="72" t="s">
+        <v>127</v>
+      </c>
+      <c r="E107" s="73" t="s">
         <v>19</v>
       </c>
-      <c r="F107" s="78"/>
-      <c r="G107" s="79"/>
-      <c r="H107" s="80">
+      <c r="F107" s="74"/>
+      <c r="G107" s="75"/>
+      <c r="H107" s="76">
         <f>'Company Definition'!N$20</f>
         <v>41.242767654986523</v>
       </c>
-      <c r="I107" s="79"/>
-      <c r="J107" s="79"/>
+      <c r="I107" s="75"/>
+      <c r="J107" s="75"/>
     </row>
     <row r="108" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B108" s="56"/>
       <c r="C108" s="56"/>
       <c r="D108" s="56" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="E108" s="55" t="s">
         <v>20</v>
@@ -4535,46 +4556,46 @@
     <row r="109" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B109" s="66"/>
       <c r="C109" s="66" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="D109" s="66"/>
       <c r="E109" s="67" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="F109" s="6">
         <v>5</v>
       </c>
       <c r="G109" s="68"/>
       <c r="H109" s="69"/>
-      <c r="I109" s="75">
+      <c r="I109" s="71">
         <f t="shared" ref="I109" si="32">(H110+H111)*F109</f>
         <v>491.74767654986522</v>
       </c>
       <c r="J109" s="68"/>
     </row>
     <row r="110" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B110" s="76"/>
-      <c r="C110" s="76"/>
-      <c r="D110" s="76" t="s">
-        <v>148</v>
-      </c>
-      <c r="E110" s="77" t="s">
+      <c r="B110" s="72"/>
+      <c r="C110" s="72"/>
+      <c r="D110" s="72" t="s">
+        <v>147</v>
+      </c>
+      <c r="E110" s="73" t="s">
         <v>19</v>
       </c>
-      <c r="F110" s="78"/>
-      <c r="G110" s="79"/>
-      <c r="H110" s="80">
+      <c r="F110" s="74"/>
+      <c r="G110" s="75"/>
+      <c r="H110" s="76">
         <f>'Company Definition'!N$20</f>
         <v>41.242767654986523</v>
       </c>
-      <c r="I110" s="79"/>
-      <c r="J110" s="79"/>
+      <c r="I110" s="75"/>
+      <c r="J110" s="75"/>
     </row>
     <row r="111" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B111" s="56"/>
       <c r="C111" s="56"/>
       <c r="D111" s="56" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="E111" s="55" t="s">
         <v>20</v>
@@ -4591,46 +4612,46 @@
     <row r="112" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B112" s="66"/>
       <c r="C112" s="66" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="D112" s="66"/>
       <c r="E112" s="67" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="F112" s="6">
         <v>6</v>
       </c>
       <c r="G112" s="68"/>
       <c r="H112" s="69"/>
-      <c r="I112" s="75">
+      <c r="I112" s="71">
         <f t="shared" ref="I112" si="33">(H113+H114)*F112</f>
         <v>590.09721185983835</v>
       </c>
       <c r="J112" s="68"/>
     </row>
     <row r="113" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B113" s="76"/>
-      <c r="C113" s="76"/>
-      <c r="D113" s="76" t="s">
-        <v>150</v>
-      </c>
-      <c r="E113" s="77" t="s">
+      <c r="B113" s="72"/>
+      <c r="C113" s="72"/>
+      <c r="D113" s="72" t="s">
+        <v>149</v>
+      </c>
+      <c r="E113" s="73" t="s">
         <v>19</v>
       </c>
-      <c r="F113" s="78"/>
-      <c r="G113" s="79"/>
-      <c r="H113" s="80">
+      <c r="F113" s="74"/>
+      <c r="G113" s="75"/>
+      <c r="H113" s="76">
         <f>'Company Definition'!N$20</f>
         <v>41.242767654986523</v>
       </c>
-      <c r="I113" s="79"/>
-      <c r="J113" s="79"/>
+      <c r="I113" s="75"/>
+      <c r="J113" s="75"/>
     </row>
     <row r="114" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B114" s="56"/>
       <c r="C114" s="56"/>
       <c r="D114" s="56" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="E114" s="55" t="s">
         <v>20</v>
@@ -4647,46 +4668,46 @@
     <row r="115" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B115" s="66"/>
       <c r="C115" s="66" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="D115" s="66"/>
       <c r="E115" s="67" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="F115" s="6">
         <v>7</v>
       </c>
       <c r="G115" s="68"/>
       <c r="H115" s="69"/>
-      <c r="I115" s="75">
+      <c r="I115" s="71">
         <f t="shared" ref="I115" si="34">(H116+H117)*F115</f>
         <v>688.44674716981137</v>
       </c>
       <c r="J115" s="68"/>
     </row>
     <row r="116" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B116" s="76"/>
-      <c r="C116" s="76"/>
-      <c r="D116" s="76" t="s">
-        <v>152</v>
-      </c>
-      <c r="E116" s="77" t="s">
+      <c r="B116" s="72"/>
+      <c r="C116" s="72"/>
+      <c r="D116" s="72" t="s">
+        <v>151</v>
+      </c>
+      <c r="E116" s="73" t="s">
         <v>19</v>
       </c>
-      <c r="F116" s="78"/>
-      <c r="G116" s="79"/>
-      <c r="H116" s="80">
+      <c r="F116" s="74"/>
+      <c r="G116" s="75"/>
+      <c r="H116" s="76">
         <f>'Company Definition'!N$20</f>
         <v>41.242767654986523</v>
       </c>
-      <c r="I116" s="79"/>
-      <c r="J116" s="79"/>
+      <c r="I116" s="75"/>
+      <c r="J116" s="75"/>
     </row>
     <row r="117" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B117" s="56"/>
       <c r="C117" s="56"/>
       <c r="D117" s="56" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="E117" s="55" t="s">
         <v>20</v>
@@ -4703,46 +4724,46 @@
     <row r="118" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B118" s="66"/>
       <c r="C118" s="66" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="D118" s="66"/>
       <c r="E118" s="67" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="F118" s="6">
         <v>8</v>
       </c>
       <c r="G118" s="68"/>
       <c r="H118" s="69"/>
-      <c r="I118" s="75">
+      <c r="I118" s="71">
         <f t="shared" ref="I118" si="35">(H119+H120)*F118</f>
         <v>786.7962824797844</v>
       </c>
       <c r="J118" s="68"/>
     </row>
     <row r="119" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B119" s="76"/>
-      <c r="C119" s="76"/>
-      <c r="D119" s="76" t="s">
-        <v>154</v>
-      </c>
-      <c r="E119" s="77" t="s">
+      <c r="B119" s="72"/>
+      <c r="C119" s="72"/>
+      <c r="D119" s="72" t="s">
+        <v>153</v>
+      </c>
+      <c r="E119" s="73" t="s">
         <v>19</v>
       </c>
-      <c r="F119" s="78"/>
-      <c r="G119" s="79"/>
-      <c r="H119" s="80">
+      <c r="F119" s="74"/>
+      <c r="G119" s="75"/>
+      <c r="H119" s="76">
         <f>'Company Definition'!N$20</f>
         <v>41.242767654986523</v>
       </c>
-      <c r="I119" s="79"/>
-      <c r="J119" s="79"/>
+      <c r="I119" s="75"/>
+      <c r="J119" s="75"/>
     </row>
     <row r="120" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B120" s="56"/>
       <c r="C120" s="56"/>
       <c r="D120" s="56" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="E120" s="55" t="s">
         <v>20</v>
@@ -4757,16 +4778,16 @@
       <c r="J120" s="54"/>
     </row>
     <row r="121" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B121" s="71" t="s">
+      <c r="B121" s="90" t="s">
         <v>16</v>
       </c>
-      <c r="C121" s="72"/>
-      <c r="D121" s="72"/>
-      <c r="E121" s="72"/>
-      <c r="F121" s="72"/>
-      <c r="G121" s="72"/>
-      <c r="H121" s="72"/>
-      <c r="I121" s="73"/>
+      <c r="C121" s="91"/>
+      <c r="D121" s="91"/>
+      <c r="E121" s="91"/>
+      <c r="F121" s="91"/>
+      <c r="G121" s="91"/>
+      <c r="H121" s="91"/>
+      <c r="I121" s="92"/>
       <c r="J121" s="59">
         <f>SUM(J4:J120)</f>
         <v>25092.629328840972</v>

</xml_diff>